<commit_message>
fix(prod): resolve recurring problem ID on Vercel with atomic sequence counter and strictly enforce production admin credentials
</commit_message>
<xml_diff>
--- a/Problem_Collector_Data.xlsx
+++ b/Problem_Collector_Data.xlsx
@@ -9,19 +9,20 @@
     <sheet sheetId="3" name="DAILY SUMMARY" state="visible" r:id="rId6"/>
     <sheet sheetId="4" name="STATUS SUMMARY" state="visible" r:id="rId7"/>
     <sheet sheetId="5" name="MONTHLY SUMMARY" state="visible" r:id="rId8"/>
-    <sheet sheetId="6" name="Education" state="visible" r:id="rId9"/>
-    <sheet sheetId="7" name="Transport" state="visible" r:id="rId10"/>
-    <sheet sheetId="8" name="Technology" state="visible" r:id="rId11"/>
-    <sheet sheetId="9" name="Food" state="visible" r:id="rId12"/>
-    <sheet sheetId="10" name="Healthcare" state="visible" r:id="rId13"/>
-    <sheet sheetId="11" name="Business" state="visible" r:id="rId14"/>
+    <sheet sheetId="6" name="Business" state="visible" r:id="rId9"/>
+    <sheet sheetId="7" name="Daily Life" state="visible" r:id="rId10"/>
+    <sheet sheetId="8" name="Healthcare" state="visible" r:id="rId11"/>
+    <sheet sheetId="9" name="Education" state="visible" r:id="rId12"/>
+    <sheet sheetId="10" name="Transport" state="visible" r:id="rId13"/>
+    <sheet sheetId="11" name="Technology" state="visible" r:id="rId14"/>
+    <sheet sheetId="12" name="Food" state="visible" r:id="rId15"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="129">
   <si>
     <t>S.No</t>
   </si>
@@ -62,39 +63,138 @@
     <t>Created At</t>
   </si>
   <si>
+    <t>ARTIX-000015</t>
+  </si>
+  <si>
+    <t>27-09-2026</t>
+  </si>
+  <si>
+    <t>11:19 PM</t>
+  </si>
+  <si>
+    <t>Business</t>
+  </si>
+  <si>
+    <t>E-commerce returns take more than two weeks for small handicraft vendors</t>
+  </si>
+  <si>
+    <t>E-commerce returns take more than two weeks for small handicraft vendors.</t>
+  </si>
+  <si>
+    <t>Business Owners</t>
+  </si>
+  <si>
+    <t>Weekly</t>
+  </si>
+  <si>
+    <t>Tirupur</t>
+  </si>
+  <si>
+    <t>Anonymous (fcff1fc9)</t>
+  </si>
+  <si>
+    <t>ACTIVE</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:49:31.468Z</t>
+  </si>
+  <si>
+    <t>ARTIX-000014</t>
+  </si>
+  <si>
+    <t>Daily Life</t>
+  </si>
+  <si>
+    <t>Electricity power fluctuations damage home refrigerators in rural subdistricts</t>
+  </si>
+  <si>
+    <t>Electricity power fluctuations damage home refrigerators in rural subdistricts.</t>
+  </si>
+  <si>
+    <t>Everyone</t>
+  </si>
+  <si>
+    <t>Daily</t>
+  </si>
+  <si>
+    <t>Salem</t>
+  </si>
+  <si>
+    <t>Anonymous (3f6b2041)</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:49:28.383Z</t>
+  </si>
+  <si>
+    <t>ARTIX-000013</t>
+  </si>
+  <si>
+    <t>Healthcare</t>
+  </si>
+  <si>
+    <t>Medical laboratory report delivery is delayed causing repeated doctor visits</t>
+  </si>
+  <si>
+    <t>Medical laboratory report delivery is delayed causing repeated doctor visits.</t>
+  </si>
+  <si>
+    <t>Senior Citizens</t>
+  </si>
+  <si>
+    <t>Madurai</t>
+  </si>
+  <si>
+    <t>Anonymous (062701d2)</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:49:25.128Z</t>
+  </si>
+  <si>
+    <t>ARTIX-000012</t>
+  </si>
+  <si>
+    <t>10:30 PM</t>
+  </si>
+  <si>
+    <t>Education</t>
+  </si>
+  <si>
+    <t>Inadequate ventilation and overcrowding in academic lecture halls affecting focus</t>
+  </si>
+  <si>
+    <t>Crowded classrooms and poor ventilation make it difficult to concentrate during afternoon lectures.</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>Coimbatore</t>
+  </si>
+  <si>
+    <t>Anonymous (user-000012)</t>
+  </si>
+  <si>
+    <t>2026-09-27T17:00:00.000Z</t>
+  </si>
+  <si>
     <t>ARTIX-000011</t>
   </si>
   <si>
-    <t>27-09-2026</t>
-  </si>
-  <si>
     <t>10:14 PM</t>
   </si>
   <si>
-    <t>Education</t>
-  </si>
-  <si>
     <t>My clg is very strict</t>
   </si>
   <si>
     <t>my clg is very strict</t>
   </si>
   <si>
-    <t>Students</t>
-  </si>
-  <si>
-    <t>Daily</t>
-  </si>
-  <si>
     <t>villupuram</t>
   </si>
   <si>
     <t>Anonymous (832eb609)</t>
   </si>
   <si>
-    <t>ACTIVE</t>
-  </si>
-  <si>
     <t>2026-09-27T16:44:41.327Z</t>
   </si>
   <si>
@@ -260,9 +360,6 @@
     <t>06:40 AM</t>
   </si>
   <si>
-    <t>Healthcare</t>
-  </si>
-  <si>
     <t>Non-transparent itemized healthcare billing and fragmented diagnostic fees.</t>
   </si>
   <si>
@@ -290,16 +387,10 @@
     <t>08:40 PM</t>
   </si>
   <si>
-    <t>Business</t>
-  </si>
-  <si>
     <t>Delayed B2B contract payouts impacting freelance cash runway.</t>
   </si>
   <si>
     <t>Clients delay invoice clearance for over 60 days leaving no cash buffer for essential operational software.</t>
-  </si>
-  <si>
-    <t>Business Owners</t>
   </si>
   <si>
     <t>Monthly</t>
@@ -763,7 +854,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:M16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -874,34 +965,34 @@
         <v>14</v>
       </c>
       <c r="D3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="H3" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="H3" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -909,40 +1000,40 @@
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>27</v>
+        <v>35</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -950,40 +1041,40 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>27</v>
+        <v>44</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>35</v>
+        <v>46</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>37</v>
+        <v>48</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M5" s="3" t="s">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -991,40 +1082,40 @@
         <v>5</v>
       </c>
       <c r="B6" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F6" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M6" s="3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1032,40 +1123,40 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>27</v>
+        <v>60</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="G7" s="4" t="s">
-        <v>54</v>
+        <v>62</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>56</v>
+        <v>64</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M7" s="3" t="s">
-        <v>57</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1073,40 +1164,40 @@
         <v>7</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E8" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="3" t="s">
-        <v>27</v>
-      </c>
       <c r="F8" s="4" t="s">
-        <v>28</v>
+        <v>61</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>36</v>
+        <v>69</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M8" s="3" t="s">
-        <v>64</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1114,40 +1205,40 @@
         <v>8</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="F9" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G9" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="H9" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>36</v>
-      </c>
       <c r="I9" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M9" s="3" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1155,40 +1246,40 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>27</v>
+        <v>80</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>36</v>
+        <v>47</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>75</v>
+        <v>55</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M10" s="3" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1196,40 +1287,40 @@
         <v>10</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>79</v>
+        <v>60</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>80</v>
+        <v>61</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>82</v>
+        <v>47</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M11" s="3" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1237,40 +1328,204 @@
         <v>11</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>89</v>
+        <v>60</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>90</v>
+        <v>61</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="H12" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J12" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="K12" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M12" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="I12" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M12" s="3" t="s">
+      <c r="D13" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>100</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J13" s="3" t="s">
         <v>95</v>
+      </c>
+      <c r="K13" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M13" s="3" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J14" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="K14" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L14" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M14" s="3" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H15" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J15" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K15" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L15" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M15" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="J16" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="K16" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M16" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -1282,7 +1537,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1346,40 +1601,245 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>77</v>
+        <v>58</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E2" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="I2" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L2" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M2" s="3" t="s">
-        <v>85</v>
+      <c r="D5" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="K5" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L6" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>107</v>
+      </c>
+      <c r="H7" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J7" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="K7" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L7" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M7" s="3" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -1455,40 +1915,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>86</v>
+        <v>77</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>88</v>
+        <v>79</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>89</v>
+        <v>80</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>93</v>
+        <v>30</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>94</v>
+        <v>55</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>63</v>
+        <v>83</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
     </row>
   </sheetData>
@@ -1498,199 +1958,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="25" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="B2" s="6">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="B3" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="B4" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="B5" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B6" s="6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="B7" s="6">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" s="6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="6">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" s="6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B5" s="6">
-        <v>1</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="20" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="6">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="18" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B2" s="6">
-        <v>11</v>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:B1"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -1756,40 +2024,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>13</v>
+        <v>98</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>14</v>
+        <v>92</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>16</v>
+        <v>100</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>17</v>
+        <v>101</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>18</v>
+        <v>102</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>19</v>
+        <v>69</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>21</v>
+        <v>95</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>22</v>
+        <v>96</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>24</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1799,9 +2067,209 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="25" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="B2" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A7" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="B7" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A8" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B8" s="6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="6">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="6">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B4" s="6">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="B5" s="6">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="20" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="6">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="24" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="B2" s="6">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -1865,22 +2333,22 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>25</v>
+        <v>13</v>
       </c>
       <c r="C2" s="2" t="s">
         <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>28</v>
+        <v>17</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>19</v>
@@ -1889,16 +2357,16 @@
         <v>20</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
@@ -1906,204 +2374,40 @@
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>33</v>
+        <v>118</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>34</v>
+        <v>120</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>28</v>
+        <v>121</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>35</v>
+        <v>122</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>20</v>
+        <v>123</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>37</v>
+        <v>124</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>38</v>
+        <v>96</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M3" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K4" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="L4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M4" s="3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J5" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M5" s="3" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J6" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="K6" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M6" s="3" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>71</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="J7" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="K7" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="M7" s="3" t="s">
-        <v>76</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -2113,7 +2417,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -2179,40 +2483,40 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>44</v>
+        <v>25</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>45</v>
+        <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>46</v>
+        <v>15</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>49</v>
+        <v>28</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>21</v>
+        <v>31</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>51</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -2222,9 +2526,9 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:M3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2288,40 +2592,231 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>65</v>
+        <v>34</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>59</v>
+        <v>14</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>66</v>
+        <v>15</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>67</v>
+        <v>35</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>68</v>
+        <v>36</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>20</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>63</v>
+        <v>40</v>
       </c>
       <c r="L2" s="2" t="s">
         <v>23</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>70</v>
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>116</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:M1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:M3"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <cols>
+    <col min="1" max="1" width="8" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="12" customWidth="1"/>
+    <col min="5" max="5" width="16" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="45" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="14" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
+    <col min="11" max="11" width="24" customWidth="1"/>
+    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="13" max="13" width="24" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="K2" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="L2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M2" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="H3" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>